<commit_message>
Judge-driven signal fixes, sleep variant, dossier, docs and workbook updates
- Critical-band rule: drone harmonics on the carriers notched; bowls moved
  to carrier-clear ratios; conch cluster at 340 Hz; chamber drone 102 Hz
  with odd harmonics; sinusoidal 40 Hz AM; unaccented drum; thunder centred.
- New 40-minute sleep variant (no call-back, no gamma, fades at the floor).
- Research dossier rebuilt from all six fact-checked lenses, three designs
  and two judges; DESIGN.md, LISTENING_GUIDE.md, README and the workbook
  updated (Sant Mat / Sikh inner-sound rows, Theosophy note, track map).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FvSmQa3U3vEBPn7cjJvA94
</commit_message>
<xml_diff>
--- a/docs/Pineal_Gateway_Breath_Protocol.xlsx
+++ b/docs/Pineal_Gateway_Breath_Protocol.xlsx
@@ -19,11 +19,11 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Protocol 48 min'!$A$3:$M$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Protocol 15 min'!$A$3:$M$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Technique Library'!$A$3:$L$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Technique Library'!$A$3:$L$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Physics &amp; Physiology'!$A$3:$F$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Goal Map'!$A$3:$G$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Playback Setup'!$A$3:$E$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Track Map'!$A$3:$I$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Track Map'!$A$3:$I$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Sources'!$A$3:$B$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -742,7 +742,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Natural breath, just observed (Anapanasati steps 1–2; Zen susokukan: count exhalations 1–10)</t>
+          <t>Natural breath, just observed (Ānāpānasati steps 1–2; Zen susokukan: count exhalations 1–10)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Return (beat 7.83 → 10 → 14.1 Hz; 963 Hz bowl at 45:20; Om bowls; tingsha)</t>
+          <t>Return (beat 7.83 → 10 → 14.1 Hz; 963 Hz bowl at 45:20; bowls on the fifth and fourth; tingsha)</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Return (call-back; 7.83 → 14.1 Hz; 963 bowl; Om bowls)</t>
+          <t>Return (call-back; 7.83 → 14.1 Hz; 963 bowl; bowls on the fifth and fourth)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
@@ -2183,7 +2183,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -5456,8 +5456,128 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="5" t="n">
+        <v>54</v>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Surat Shabd Yoga (Sant Mat: Radha Soami, Ruhani Satsang, Kirpal Singh, Sawan Singh)</t>
+        </is>
+      </c>
+      <c r="C57" s="5" t="inlineStr">
+        <is>
+          <t>Sant Mat lineages (Shiv Dayal Singh, 1861 →); taught by initiation (naam-daan) with a vow of 2.5 h daily practice</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Initiatory (the five charged names are given at initiation); the method is described in public books (Julian Johnson, The Path of the Masters 1939; Sawan Singh, Philosophy of the Masters)</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Two parts: simran (silent repetition of the charged names with attention held at the 'eye centre' between and behind the eyebrows, ~2 h) and bhajan (sitting with the thumbs closing the ears, listening for the inner sound current — bell, conch, flute, harp-like sounds — and following the subtlest one upward; ~30 min). Breath is not controlled; the body is forgotten.</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>natural</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>Seated, often with the elbows on a bhajan stick</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>The soul (surat) attaches to the sound current (shabd) and travels through the inner regions (Sahansdal Kanwal, Trikuti, Daswan Dwar, Bhanwar Gupha, Sach Khand); the explicit doctrine of leaving the body and ascending realms by sound.</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Attention withdrawn to one point plus ear closure: the same absorption-and-otoacoustic/inner-noise mechanism as nāda anusandhāna (#14), framed as ascent.</t>
+        </is>
+      </c>
+      <c r="J57" s="5" t="inlineStr">
+        <is>
+          <t>Traditional.</t>
+        </is>
+      </c>
+      <c r="K57" s="5" t="inlineStr">
+        <is>
+          <t>The No-Time stage listening posture; the Crown stage; the workbook's inner-sound rows.</t>
+        </is>
+      </c>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Naam Simran and the anhad shabad (Sikh)</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>Sikh practice (Guru Granth Sahib; Bhai Randhir Singh, Anhad Shabad Dasam Duar)</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>Public</t>
+        </is>
+      </c>
+      <c r="E58" s="4" t="inlineStr">
+        <is>
+          <t>Repetition of 'Waheguru' on the breath ('Wahe' in, 'Guru' out) or the Mul Mantar, in the ambrosial hours (amrit vela, ~3–6 a.m.), for 30 min to hours; the unstruck sound (anhad shabad) and the nectar (amrit) are described as the signs of the tenth gate (dasam duar) opening.</t>
+        </is>
+      </c>
+      <c r="F58" s="4" t="inlineStr">
+        <is>
+          <t>natural (4–6 s cycle)</t>
+        </is>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>Seated</t>
+        </is>
+      </c>
+      <c r="H58" s="4" t="inlineStr">
+        <is>
+          <t>Union with the Name; the tenth gate opens; the celestial kirtan is heard. The tradition explicitly rejects seeking powers.</t>
+        </is>
+      </c>
+      <c r="I58" s="4" t="inlineStr">
+        <is>
+          <t>Breath-linked mantra at the coherent rate (as #13, #42).</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="inlineStr">
+        <is>
+          <t>Traditional.</t>
+        </is>
+      </c>
+      <c r="K58" s="4" t="inlineStr">
+        <is>
+          <t>Descent (as the breath anchor) and the early-morning timing option.</t>
+        </is>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:L56"/>
+  <autoFilter ref="A3:L58"/>
   <mergeCells count="1">
     <mergeCell ref="A2:L2"/>
   </mergeCells>
@@ -7119,7 +7239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -7227,7 +7347,7 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Tingsha, bonshō, tanpura Om drone (136.1 + 204.15), Om bowls (wah at 8 Hz, right-leaning), breath pacer 8 → 6/min, pink bed</t>
+          <t>Tingsha, bonshō, tanpura Om drone (136.1 + 204.15 Pa string), bowls on the fifth and fourth (204 / 181 Hz, wah at 8 Hz, right-leaning), breath pacer 8 → 6/min, pink bed</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
@@ -7274,7 +7394,7 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Gyuto chord drone 68.05 Hz (5th/10th harmonics), bowls 204 &amp; 272 Hz (wah 7.83), dungchen 9:18, pacer 6/min</t>
+          <t>Gyuto chord drone 68.05 Hz (5th/10th harmonics), bowls 204 &amp; 340 Hz (wah 7.83), dungchen 9:18, pacer 6/min</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
@@ -7316,12 +7436,12 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Frame drum 4.25 Hz 11:30–20:30; theta isochronic 204 Hz 12:30–21:30</t>
+          <t>Frame drum 4.25 Hz 11:30–20:30 (unaccented); theta isochronic 204 Hz 12:30–21:30</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Thunder 10:54, didgeridoo 68 Hz with 0.55 Hz breath pulse, chamber drone 108.9 Hz (reverberant), bowls 136 &amp; 204 (wah 4.25)</t>
+          <t>Thunder 10:54, didgeridoo 68 Hz with 0.55 Hz breath pulse, chamber drone 102 Hz (odd harmonics, reverberant), bowls 181 &amp; 204 (wah 4.25)</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
@@ -7368,12 +7488,12 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Seven-vowel choir A E Ē I O U Ō rising 136 → 255 Hz then IAŌ; chakra bowl ladder 272 → 510 Hz (wah 6 Hz)</t>
+          <t>Seven-vowel choir A E Ē I O U Ō rising 136 → 255 Hz then IAŌ; seven-bowl ascent 181 → 817 Hz (4:3, 3:2, 5:2, 15:4, 9:2, 5:1, 6:1; wah 6 Hz)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Greek Magical Papyri / Shat-chakra-nirupana / Goldman</t>
+          <t>Greek Magical Papyri / Shat-chakra-nirupana / Goldman (model)</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
@@ -7410,12 +7530,12 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>Theta isochronic 29:30–37:00; 40 Hz cues at 31:48, 34:18, 36:36</t>
+          <t>Theta isochronic 29:30–37:00; 40 Hz sinusoidal-AM cues at 31:48, 34:18, 36:36</t>
         </is>
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Dungchen 30:00/33:30/36:00, bowls 136 (3 Hz) &amp; 272 (2.13 Hz), 0.2 Hz surge on the drone, thunders 35:24–36:30</t>
+          <t>Dungchen 30:00/33:30/36:00, bowls 181 (3 Hz) &amp; 340 (2.13 Hz), 0.2 Hz surge on the drone, thunders 35:24–36:30</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
@@ -7462,7 +7582,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>A-OM-HUM choir (272/204/136 Hz), Gyuto drone, pututu conch clusters 38:36/40:24/42:00, bowls 272/408/544/136, 3–8 kHz air</t>
+          <t>A-OM-HUM choir (272/204/136 Hz), Gyuto drone, pututu conch clusters at 340 Hz 38:36/40:24/42:00, bowls 340/510/680/204, 3–8 kHz air</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
@@ -7494,12 +7614,12 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>7.83 → 10 (45:30) → 14.1 (47:30)</t>
+          <t>7.83 → 10 (45:18) → 14.1 (47:36)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>7.83 → 14.1</t>
+          <t>7.83 (to 46:00) → 12.5</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -7509,7 +7629,7 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>963 Hz bowl 45:20 (alone), Om bowls 46:00/46:48/47:30 (wah 10 Hz), pacer 6 → 7/min, tingsha 47:50</t>
+          <t>963 Hz bowl 45:20 (alone), bowls 204/181/204 at 46:00/46:48/47:30 (wah 10 Hz), pacer 6 → 7/min, tingsha 47:50</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
@@ -7523,8 +7643,55 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Sleep variant (40 min)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>as above to 2.13 Hz at 34:30, then held</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>10 to 35:00, then 2.13</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Theta isochronic to 37:00; no 40 Hz</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>Full arc to the floor; no call-back, thunders or conch; everything fades 36:30–39:30</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t>Focus 15 / Yoga Nidra sleep</t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>Let go</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:I10"/>
+  <autoFilter ref="A3:I11"/>
   <mergeCells count="1">
     <mergeCell ref="A2:I2"/>
   </mergeCells>

</xml_diff>